<commit_message>
major update on place
</commit_message>
<xml_diff>
--- a/userProfile/instapay_template.xlsx
+++ b/userProfile/instapay_template.xlsx
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="D5" s="19" t="n"/>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>1+admin1</t>
         </is>
@@ -1733,22 +1733,48 @@
     <row r="6" ht="15.75" customHeight="1" s="24">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Select Bank…</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
+          <t>Bangko Mabuhay (A Rural Bank), Inc.</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>jojo</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="D6" s="19" t="n"/>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>26+popo</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="24">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Select Bank…</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="n"/>
-      <c r="C7" s="19" t="n"/>
+          <t>Alipay Philippines</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>asdasdasdasdad asda sd</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>123123123123123123</t>
+        </is>
+      </c>
       <c r="D7" s="19" t="n"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>26+popo</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="24">
       <c r="A8" s="16" t="inlineStr">

</xml_diff>